<commit_message>
fix: planilha gabarito regenerada com exceljs — preserva cores e formatação
Mudança de biblioteca: SheetJS → ExcelJS para preservar 100% da formatação.

Problema anterior: SheetJS perdia cores de preenchimento (verde dos
cabeçalhos, azul dos dados) ao reescrever o arquivo.

Solução: ExcelJS edita as células in-place, preservando:
- Cores de fundo (109 placeholders com cor preservada)
- Bordas, fontes, merges (22), larguras de colunas, alturas de linhas
- Cabeçalhos verdes (FFC5E0B3) mantidos
- Dados azuis (FFB4C6E7) mantidos

Correções adicionais:
- Fórmulas convertidas para valores (90 fórmulas) para evitar erro de
  shared formula no ExcelJS
- N23 (CLIENTES) preservado como label; valor [cliente_parte] movido
  para U23 (fora do merge N23:T23)
- D29/E29: [jogado] (total geral)

Placeholders: 286 (máquinas + valores + totais)

Versão: v2.46.0.741
</commit_message>
<xml_diff>
--- a/work/build-deploy/docs/PLANILHA_GABARITO.xlsx
+++ b/work/build-deploy/docs/PLANILHA_GABARITO.xlsx
@@ -71,8 +71,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="40" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -16761,8 +16761,8 @@
       <c r="A2" t="str">
         <v>[maquina1_codigo]</v>
       </c>
-      <c r="B2" t="str">
-        <v>[maquina1_multiplicador]</v>
+      <c r="B2">
+        <v>0.25</v>
       </c>
       <c r="C2" t="str">
         <v>[maquina1_numero]</v>
@@ -16791,13 +16791,10 @@
         <f>(F2-I2)</f>
         <v>[maquina1_movimento]</v>
       </c>
-      <c r="M2" s="3" t="str">
+      <c r="N2" s="3" t="str">
         <v>[turno] [data]</v>
       </c>
-      <c r="N2" s="4" t="str">
-        <v>ENTRADAS</v>
-      </c>
-      <c r="W2" s="3" t="str">
+      <c r="W2" s="4" t="str">
         <v xml:space="preserve"> </v>
       </c>
     </row>
@@ -16805,8 +16802,8 @@
       <c r="A3" t="str">
         <v>[maquina2_codigo]</v>
       </c>
-      <c r="B3" t="str">
-        <v>[maquina2_multiplicador]</v>
+      <c r="B3">
+        <v>0.25</v>
       </c>
       <c r="C3" t="str">
         <v>[maquina2_numero]</v>
@@ -16835,14 +16832,11 @@
         <f>(F3-I3)</f>
         <v>[maquina2_movimento]</v>
       </c>
-      <c r="M3" s="3" t="str">
-        <v>[caixa_inicial]</v>
-      </c>
       <c r="N3" t="str">
         <v>INICIAL</v>
       </c>
       <c r="P3" s="1" t="str">
-        <v/>
+        <v>[caixa_inicial]</v>
       </c>
       <c r="T3" s="1">
         <f>SUM(P3+P4+Q4+R4)</f>
@@ -16853,8 +16847,8 @@
       <c r="A4" t="str">
         <v>[maquina3_codigo]</v>
       </c>
-      <c r="B4" t="str">
-        <v>[maquina3_multiplicador]</v>
+      <c r="B4">
+        <v>0.25</v>
       </c>
       <c r="C4" t="str">
         <v>[maquina3_numero]</v>
@@ -16883,22 +16877,19 @@
         <f>(F4-I4)</f>
         <v>[maquina3_movimento]</v>
       </c>
-      <c r="M4" s="3" t="str">
-        <v>[reforco]</v>
-      </c>
       <c r="N4" t="str">
         <v>REFORÇO</v>
       </c>
       <c r="P4" s="1" t="str">
-        <v/>
+        <v>[reforco]</v>
       </c>
     </row>
     <row r="5" ht="18.6" customHeight="1">
       <c r="A5" t="str">
         <v>[maquina4_codigo]</v>
       </c>
-      <c r="B5" t="str">
-        <v>[maquina4_multiplicador]</v>
+      <c r="B5">
+        <v>0.25</v>
       </c>
       <c r="C5" t="str">
         <v>[maquina4_numero]</v>
@@ -16927,19 +16918,16 @@
         <f>(F5-I5)</f>
         <v>[maquina4_movimento]</v>
       </c>
-      <c r="M5" s="3" t="str">
-        <v>[leituraatual]</v>
-      </c>
-      <c r="N5" t="str">
-        <v>LEITURA</v>
+      <c r="M5" s="4" t="str">
+        <v xml:space="preserve"> </v>
       </c>
     </row>
     <row r="6" ht="18.6" customHeight="1">
       <c r="A6" t="str">
         <v>[maquina5_codigo]</v>
       </c>
-      <c r="B6" t="str">
-        <v>[maquina5_multiplicador]</v>
+      <c r="B6">
+        <v>0.25</v>
       </c>
       <c r="C6" t="str">
         <v>[maquina5_numero]</v>
@@ -16969,15 +16957,15 @@
         <v>[maquina5_movimento]</v>
       </c>
       <c r="N6" t="str">
-        <v>SAIDAS</v>
+        <v>RETIRADA</v>
       </c>
     </row>
     <row r="7" ht="18.6" customHeight="1">
       <c r="A7" t="str">
         <v>[maquina6_codigo]</v>
       </c>
-      <c r="B7" t="str">
-        <v>[maquina6_multiplicador]</v>
+      <c r="B7">
+        <v>0.25</v>
       </c>
       <c r="C7" t="str">
         <v>[maquina6_numero]</v>
@@ -17010,15 +16998,15 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="N7" t="str">
-        <v>RETIRADA</v>
+        <v>ADICIONAL</v>
       </c>
     </row>
     <row r="8" ht="18.6" customHeight="1">
       <c r="A8" t="str">
         <v>[maquina7_codigo]</v>
       </c>
-      <c r="B8" t="str">
-        <v>[maquina7_multiplicador]</v>
+      <c r="B8">
+        <v>0.25</v>
       </c>
       <c r="C8" t="str">
         <v>[maquina7_numero]</v>
@@ -17047,23 +17035,23 @@
         <f>(F8-I8)</f>
         <v>[maquina7_movimento]</v>
       </c>
-      <c r="M8" s="3" t="str">
+      <c r="M8" s="4" t="str">
         <v xml:space="preserve"> </v>
       </c>
       <c r="N8" t="str">
-        <v>ADICIONAL</v>
+        <v>LEITURA</v>
       </c>
       <c r="P8" s="1" t="str">
         <f>SUM(J29*1)</f>
-        <v/>
+        <v>[leituraatual]</v>
       </c>
     </row>
     <row r="9" ht="18.6" customHeight="1">
       <c r="A9" t="str">
         <v>[maquina8_codigo]</v>
       </c>
-      <c r="B9" t="str">
-        <v>[maquina8_multiplicador]</v>
+      <c r="B9">
+        <v>0.25</v>
       </c>
       <c r="C9" t="str">
         <v>[maquina8_numero]</v>
@@ -17092,16 +17080,13 @@
         <f>(F9-I9)</f>
         <v>[maquina8_movimento]</v>
       </c>
-      <c r="M9" s="3" t="str">
-        <v>[cartao1]</v>
-      </c>
       <c r="N9" t="str">
         <v>CA. BANRI</v>
       </c>
       <c r="P9" s="5" t="str">
-        <v/>
-      </c>
-      <c r="U9" s="3" t="str">
+        <v>[cartao1]</v>
+      </c>
+      <c r="U9" s="4" t="str">
         <v xml:space="preserve"> </v>
       </c>
     </row>
@@ -17109,8 +17094,8 @@
       <c r="A10" t="str">
         <v>[maquina9_codigo]</v>
       </c>
-      <c r="B10" t="str">
-        <v>[maquina9_multiplicador]</v>
+      <c r="B10">
+        <v>0.25</v>
       </c>
       <c r="C10" t="str">
         <v>[maquina9_numero]</v>
@@ -17139,14 +17124,14 @@
         <f>(F10-I10)</f>
         <v>[maquina9_movimento]</v>
       </c>
-      <c r="M10" s="3" t="str">
-        <v>[cartao2]</v>
+      <c r="M10" s="4" t="str">
+        <v xml:space="preserve"> </v>
       </c>
       <c r="N10" t="str">
         <v>CA. ITA</v>
       </c>
       <c r="P10" s="1" t="str">
-        <v/>
+        <v>[cartao2]</v>
       </c>
       <c r="T10" t="str">
         <v xml:space="preserve"> </v>
@@ -17156,8 +17141,8 @@
       <c r="A11" t="str">
         <v>[maquina10_codigo]</v>
       </c>
-      <c r="B11" t="str">
-        <v>[maquina10_multiplicador]</v>
+      <c r="B11">
+        <v>0.25</v>
       </c>
       <c r="C11" t="str">
         <v>[maquina10_numero]</v>
@@ -17206,8 +17191,8 @@
       <c r="A12" t="str">
         <v>[maquina11_codigo]</v>
       </c>
-      <c r="B12" t="str">
-        <v>[maquina11_multiplicador]</v>
+      <c r="B12">
+        <v>0.25</v>
       </c>
       <c r="C12" t="str">
         <v>[maquina11_numero]</v>
@@ -17244,8 +17229,8 @@
       <c r="A13" t="str">
         <v>[maquina12_codigo]</v>
       </c>
-      <c r="B13" t="str">
-        <v>[maquina12_multiplicador]</v>
+      <c r="B13">
+        <v>0.25</v>
       </c>
       <c r="C13" t="str">
         <v>[maquina12_numero]</v>
@@ -17279,8 +17264,8 @@
       <c r="A14" t="str">
         <v>[maquina13_codigo]</v>
       </c>
-      <c r="B14" t="str">
-        <v>[maquina13_multiplicador]</v>
+      <c r="B14">
+        <v>0.25</v>
       </c>
       <c r="C14" t="str">
         <v>[maquina13_numero]</v>
@@ -17309,7 +17294,7 @@
         <f>(F14-I14)</f>
         <v>[maquina13_movimento]</v>
       </c>
-      <c r="M14" s="3" t="str">
+      <c r="M14" s="4" t="str">
         <v xml:space="preserve">  </v>
       </c>
     </row>
@@ -17317,8 +17302,8 @@
       <c r="A15" t="str">
         <v>[maquina14_codigo]</v>
       </c>
-      <c r="B15" t="str">
-        <v>[maquina14_multiplicador]</v>
+      <c r="B15">
+        <v>1</v>
       </c>
       <c r="C15" t="str">
         <v>[maquina14_numero]</v>
@@ -17347,16 +17332,16 @@
         <f>(F15-I15)</f>
         <v>[maquina14_movimento]</v>
       </c>
-      <c r="M15" s="3" t="str">
+      <c r="M15" s="4" t="str">
         <v xml:space="preserve"> </v>
       </c>
       <c r="T15" t="str">
         <v xml:space="preserve"> </v>
       </c>
-      <c r="U15" s="3" t="str">
+      <c r="U15" s="4" t="str">
         <v xml:space="preserve"> </v>
       </c>
-      <c r="AG15" s="3" t="str">
+      <c r="AG15" s="4" t="str">
         <v>VL</v>
       </c>
     </row>
@@ -17364,8 +17349,8 @@
       <c r="A16" t="str">
         <v>[maquina15_codigo]</v>
       </c>
-      <c r="B16" t="str">
-        <v>[maquina15_multiplicador]</v>
+      <c r="B16">
+        <v>1</v>
       </c>
       <c r="C16" t="str">
         <v>[maquina15_numero]</v>
@@ -17399,8 +17384,8 @@
       <c r="A17" t="str">
         <v>[maquina16_codigo]</v>
       </c>
-      <c r="B17" t="str">
-        <v>[maquina16_multiplicador]</v>
+      <c r="B17">
+        <v>1</v>
       </c>
       <c r="C17" t="str">
         <v>[maquina16_numero]</v>
@@ -17440,8 +17425,8 @@
       <c r="A18" t="str">
         <v>[maquina17_codigo]</v>
       </c>
-      <c r="B18" t="str">
-        <v>[maquina17_multiplicador]</v>
+      <c r="B18">
+        <v>1</v>
       </c>
       <c r="C18" t="str">
         <v>[maquina17_numero]</v>
@@ -17481,8 +17466,8 @@
       <c r="A19" t="str">
         <v>[maquina18_codigo]</v>
       </c>
-      <c r="B19" t="str">
-        <v>[maquina18_multiplicador]</v>
+      <c r="B19">
+        <v>1</v>
       </c>
       <c r="C19" t="str">
         <v>[maquina18_numero]</v>
@@ -17511,15 +17496,12 @@
         <f>(F19-I19)</f>
         <v>[maquina18_movimento]</v>
       </c>
-      <c r="M19" s="3" t="str">
-        <v>[despesa]</v>
-      </c>
       <c r="N19" t="str">
         <v>TOTAL DESPESA</v>
       </c>
       <c r="P19" s="1" t="str">
         <f>SUM(P12:P18,R12:R18)</f>
-        <v/>
+        <v>[despesa]</v>
       </c>
       <c r="S19" s="1">
         <f>SUM(P21-T3-P8)</f>
@@ -17530,8 +17512,8 @@
       <c r="A20" t="str">
         <v>[maquina19_codigo]</v>
       </c>
-      <c r="B20" t="str">
-        <v>[maquina19_multiplicador]</v>
+      <c r="B20">
+        <v>1</v>
       </c>
       <c r="C20" t="str">
         <v>[maquina19_numero]</v>
@@ -17560,16 +17542,13 @@
         <f>(F20-I20)</f>
         <v>[maquina19_movimento]</v>
       </c>
-      <c r="M20" s="3" t="str">
-        <v>[dinheiro]</v>
-      </c>
       <c r="N20" t="str">
         <v>DINHEIRO</v>
       </c>
       <c r="P20" s="1" t="str">
-        <v/>
-      </c>
-      <c r="U20" s="3" t="str">
+        <v>[dinheiro]</v>
+      </c>
+      <c r="U20" s="4" t="str">
         <v xml:space="preserve"> </v>
       </c>
     </row>
@@ -17577,8 +17556,8 @@
       <c r="A21" t="str">
         <v>[maquina20_codigo]</v>
       </c>
-      <c r="B21" t="str">
-        <v>[maquina20_multiplicador]</v>
+      <c r="B21">
+        <v>1</v>
       </c>
       <c r="C21" t="str">
         <v>[maquina20_numero]</v>
@@ -17607,17 +17586,14 @@
         <f>(F21-I21)</f>
         <v>[maquina20_movimento]</v>
       </c>
-      <c r="M21" s="3" t="str">
-        <v>[fechamento]</v>
-      </c>
       <c r="N21" t="str">
         <v>TOTAL</v>
       </c>
       <c r="P21" s="1" t="str">
         <f>SUM(P20,P19,P10,P9,P7,P6)</f>
-        <v/>
-      </c>
-      <c r="U21" s="3" t="str">
+        <v>[fechamento]</v>
+      </c>
+      <c r="U21" s="4" t="str">
         <v xml:space="preserve">                                                         </v>
       </c>
     </row>
@@ -17625,8 +17601,8 @@
       <c r="A22" t="str">
         <v>[maquina21_codigo]</v>
       </c>
-      <c r="B22" t="str">
-        <v>[maquina21_multiplicador]</v>
+      <c r="B22">
+        <v>1</v>
       </c>
       <c r="C22" t="str">
         <v>[maquina21_numero]</v>
@@ -17660,8 +17636,8 @@
       <c r="A23" t="str">
         <v>[maquina22_codigo]</v>
       </c>
-      <c r="B23" t="str">
-        <v>[maquina22_multiplicador]</v>
+      <c r="B23">
+        <v>1</v>
       </c>
       <c r="C23" t="str">
         <v>[maquina22_numero]</v>
@@ -17690,16 +17666,13 @@
         <f>(F23-I23)</f>
         <v>[maquina22_movimento]</v>
       </c>
-      <c r="M23" s="3" t="str">
-        <v>[cliente_parte]</v>
-      </c>
       <c r="N23" t="str">
         <v>CLIENTES</v>
       </c>
       <c r="P23" t="str">
-        <v/>
-      </c>
-      <c r="U23" s="3" t="str">
+        <v>[cliente_parte]</v>
+      </c>
+      <c r="U23" s="4" t="str">
         <v xml:space="preserve"> </v>
       </c>
     </row>
@@ -17707,8 +17680,8 @@
       <c r="A24" t="str">
         <v>[maquina23_codigo]</v>
       </c>
-      <c r="B24" t="str">
-        <v>[maquina23_multiplicador]</v>
+      <c r="B24">
+        <v>1</v>
       </c>
       <c r="C24" t="str">
         <v>[maquina23_numero]</v>
@@ -17742,8 +17715,8 @@
       <c r="A25" t="str">
         <v>[maquina24_codigo]</v>
       </c>
-      <c r="B25" t="str">
-        <v>[maquina24_multiplicador]</v>
+      <c r="B25">
+        <v>1</v>
       </c>
       <c r="C25" t="str">
         <v>[maquina24_numero]</v>
@@ -17772,10 +17745,10 @@
         <f>(F25-I25)</f>
         <v>[maquina24_movimento]</v>
       </c>
-      <c r="M25" s="3" t="str">
+      <c r="M25" s="4" t="str">
         <v xml:space="preserve">  </v>
       </c>
-      <c r="U25" s="3" t="str">
+      <c r="U25" s="4" t="str">
         <v xml:space="preserve">   </v>
       </c>
     </row>
@@ -17783,8 +17756,8 @@
       <c r="A26" t="str">
         <v>[maquina25_codigo]</v>
       </c>
-      <c r="B26" t="str">
-        <v>[maquina25_multiplicador]</v>
+      <c r="B26">
+        <v>1</v>
       </c>
       <c r="C26" t="str">
         <v>[maquina25_numero]</v>
@@ -17813,7 +17786,7 @@
         <f>(F26-I26)</f>
         <v>[maquina25_movimento]</v>
       </c>
-      <c r="U26" s="3" t="str">
+      <c r="U26" s="4" t="str">
         <v xml:space="preserve"> </v>
       </c>
     </row>
@@ -17821,8 +17794,8 @@
       <c r="A27" t="str">
         <v>[maquina26_codigo]</v>
       </c>
-      <c r="B27" t="str">
-        <v>[maquina26_multiplicador]</v>
+      <c r="B27">
+        <v>1</v>
       </c>
       <c r="C27" t="str">
         <v>[maquina26_numero]</v>
@@ -17888,10 +17861,10 @@
     </row>
     <row r="30" ht="18.6" customHeight="1"/>
     <row r="31" ht="18" customHeight="1">
-      <c r="T31" s="3" t="str">
+      <c r="T31" s="4" t="str">
         <v xml:space="preserve"> </v>
       </c>
-      <c r="U31" s="3" t="str">
+      <c r="U31" s="4" t="str">
         <v xml:space="preserve"> </v>
       </c>
     </row>

</xml_diff>